<commit_message>
per utenti non abilitati, nak sulla useEffect
per evitare di far riempire tutta la form e avere errore solo alla submit
</commit_message>
<xml_diff>
--- a/src/frontend/prepare_i18n/dossier.xlsx
+++ b/src/frontend/prepare_i18n/dossier.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="265">
   <si>
     <t xml:space="preserve">L1</t>
   </si>
@@ -196,132 +196,6 @@
     <t xml:space="preserve">Nessun Documento Presente</t>
   </si>
   <si>
-    <t xml:space="preserve">mimetype</t>
-  </si>
-  <si>
-    <t xml:space="preserve">image/jpeg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jpeg image</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Immagine jpeg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">application/pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PDF document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documento PDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">application/vndopenxmlformats-officedocumentwordprocessingmldocument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Word document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documento word</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tiposupporto_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP_TELA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Canvas, paper, wood, fabric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela, carta, legno, stoffa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP_PLASTICA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plastic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plastica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP_METALLO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metallo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP_DIGITAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital image</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Immagine digitale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP_OTHER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altri supporti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">statusopera_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS_AVAILABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Available</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disponibile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS_RESTORATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Under restoration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Restauro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS_ON_LOAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Borrowed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Prestito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS_DESTROYED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Destroyed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distrutta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS_STOLEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stolen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rubata</t>
-  </si>
-  <si>
     <t xml:space="preserve">Altro</t>
   </si>
   <si>
@@ -337,63 +211,6 @@
     <t xml:space="preserve">Fruibilita Dossier</t>
   </si>
   <si>
-    <t xml:space="preserve">fruibilitadossier_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_COMPLETELY_PRIVATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completely private</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completamente privato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_COMPLETELY_RESERVED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completely confidential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completamente riservato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_TASSONOMICALLY_RESERVED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserved for Taxonomy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riservato per Tassonomia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_SINGLE_DOCUMENT_RESERVED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserved for single document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riservato per singolo documento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_TASSONOMICALLY_PUBLIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public by taxonomy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pubblico per tassonomia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOSSIER_FRUIBILITY_COMPLETELY_PUBLIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completely public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completamente pubblico</t>
-  </si>
-  <si>
     <t xml:space="preserve">FruibilitaOpera</t>
   </si>
   <si>
@@ -403,84 +220,12 @@
     <t xml:space="preserve">Fruibilita Opera</t>
   </si>
   <si>
-    <t xml:space="preserve">fruibilitaopera_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPERA_FRUIBILITY_PRIVATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Private</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Privata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPERA_FRUIBILITY_PUBLIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exhibited to the public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esposta al Pubblico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPERA_FRUIBILITY_ON_REQUEST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visible by appointment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visibile su Appuntamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tipoluogo_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUOGO_MUSEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Museum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Museo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUOGO_COLLEZIONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collezione</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUOGO_GALLERIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gallery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Galleria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUOGO_PROPRIETARIO</t>
+    <t xml:space="preserve">Proprietario</t>
   </si>
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">Proprietario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUOGO_SCONOSCIUTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sconosciuto</t>
-  </si>
-  <si>
     <t xml:space="preserve">Documenti</t>
   </si>
   <si>
@@ -1052,6 +797,24 @@
   </si>
   <si>
     <t xml:space="preserve">I documenti possono essere associati solo alla copia principale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">view_opera_nak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You are not entitled to view operas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non hai i diritti per visualizzare le opere</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add_opera_nak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You are not entitled to add operas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non hai i diritti per aggiungere opere</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +824,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1083,6 +846,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1127,12 +896,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1153,11 +926,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D132"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D1048576"/>
+  <sheetFormatPr defaultColWidth="8.9140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54.23"/>
   </cols>
@@ -1422,412 +1195,448 @@
       <c r="A24" s="0" t="s">
         <v>58</v>
       </c>
+      <c r="C24" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0" t="s">
-        <v>59</v>
+      <c r="A25" s="0" t="s">
+        <v>60</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0" t="s">
-        <v>62</v>
+      <c r="A26" s="0" t="s">
+        <v>63</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="0" t="s">
-        <v>65</v>
+      <c r="A27" s="0" t="s">
+        <v>66</v>
       </c>
       <c r="C27" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="0" t="s">
         <v>66</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
         <v>68</v>
       </c>
+      <c r="C28" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="0" t="s">
-        <v>69</v>
+      <c r="A29" s="0" t="s">
+        <v>70</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="0" t="s">
-        <v>72</v>
+      <c r="A30" s="0" t="s">
+        <v>73</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0" t="s">
-        <v>75</v>
+      <c r="A31" s="0" t="s">
+        <v>76</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="0" t="s">
-        <v>78</v>
+      <c r="A32" s="0" t="s">
+        <v>79</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0" t="s">
-        <v>81</v>
+      <c r="A33" s="0" t="s">
+        <v>82</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="0" t="s">
-        <v>85</v>
+      <c r="A35" s="0" t="s">
+        <v>88</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="0" t="s">
-        <v>88</v>
+      <c r="A36" s="0" t="s">
+        <v>91</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>89</v>
+        <v>25</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="0" t="s">
-        <v>91</v>
+      <c r="A37" s="0" t="s">
+        <v>92</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="0" t="s">
-        <v>94</v>
+      <c r="A38" s="0" t="s">
+        <v>95</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="0" t="s">
-        <v>97</v>
+      <c r="A39" s="0" t="s">
+        <v>98</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C40" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="D40" s="0" t="s">
         <v>101</v>
-      </c>
-      <c r="D40" s="0" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="0" t="s">
-        <v>106</v>
+      <c r="A43" s="0" t="s">
+        <v>109</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="0" t="s">
-        <v>109</v>
+      <c r="A44" s="0" t="s">
+        <v>112</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="0" t="s">
-        <v>112</v>
+      <c r="A45" s="0" t="s">
+        <v>115</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="0" t="s">
-        <v>115</v>
+      <c r="A46" s="0" t="s">
+        <v>117</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D46" s="0" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="0" t="s">
-        <v>118</v>
+      <c r="A47" s="0" t="s">
+        <v>119</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="0" t="s">
-        <v>121</v>
+      <c r="A48" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
+      </c>
+      <c r="C50" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="D50" s="0" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="0" t="s">
-        <v>128</v>
+      <c r="A51" s="0" t="s">
+        <v>131</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="0" t="s">
-        <v>131</v>
+      <c r="A52" s="0" t="s">
+        <v>134</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="0" t="s">
-        <v>134</v>
+      <c r="A53" s="0" t="s">
+        <v>137</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>137</v>
+        <v>140</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="D54" s="0" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="0" t="s">
-        <v>138</v>
+      <c r="A55" s="0" t="s">
+        <v>143</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="0" t="s">
-        <v>141</v>
+      <c r="A56" s="0" t="s">
+        <v>146</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="0" t="s">
-        <v>144</v>
+      <c r="A57" s="0" t="s">
+        <v>148</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="0" t="s">
-        <v>147</v>
+      <c r="A58" s="0" t="s">
+        <v>151</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="0" t="s">
-        <v>150</v>
+      <c r="A59" s="0" t="s">
+        <v>153</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D64" s="0" t="s">
         <v>163</v>
@@ -1835,10 +1644,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D65" s="0" t="s">
         <v>166</v>
@@ -1852,40 +1661,40 @@
         <v>168</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="C67" s="0" t="s">
         <v>170</v>
       </c>
-      <c r="C67" s="0" t="s">
-        <v>171</v>
-      </c>
       <c r="D67" s="0" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="D68" s="0" t="s">
         <v>173</v>
-      </c>
-      <c r="C68" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="D68" s="0" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="D69" s="0" t="s">
         <v>176</v>
-      </c>
-      <c r="C69" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1929,51 +1738,51 @@
         <v>187</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C77" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="D77" s="0" t="s">
         <v>198</v>
-      </c>
-      <c r="D77" s="0" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1984,26 +1793,26 @@
         <v>201</v>
       </c>
       <c r="D78" s="0" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D79" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D80" s="0" t="s">
         <v>206</v>
@@ -2011,13 +1820,13 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C81" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="D81" s="0" t="s">
         <v>208</v>
-      </c>
-      <c r="D81" s="0" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2028,114 +1837,114 @@
         <v>211</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="C83" s="0" t="s">
         <v>213</v>
       </c>
-      <c r="C83" s="0" t="s">
-        <v>214</v>
-      </c>
       <c r="D83" s="0" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="C84" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="D84" s="0" t="s">
         <v>216</v>
-      </c>
-      <c r="C84" s="0" t="s">
-        <v>217</v>
-      </c>
-      <c r="D84" s="0" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D85" s="0" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D86" s="0" t="s">
-        <v>224</v>
+        <v>197</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D87" s="0" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="C88" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="D88" s="0" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="C89" s="0" t="s">
         <v>228</v>
       </c>
-      <c r="C88" s="0" t="s">
+      <c r="D89" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="D88" s="0" t="s">
+    </row>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="0" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0" t="s">
+      <c r="C90" s="0" t="s">
         <v>231</v>
       </c>
-      <c r="C89" s="0" t="s">
+      <c r="D90" s="1" t="s">
         <v>232</v>
-      </c>
-      <c r="D89" s="0" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0" t="s">
-        <v>233</v>
-      </c>
-      <c r="C90" s="0" t="s">
-        <v>234</v>
-      </c>
-      <c r="D90" s="0" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C91" s="0" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D91" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D92" s="0" t="s">
         <v>238</v>
@@ -2143,444 +1952,136 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="C93" s="0" t="s">
         <v>240</v>
       </c>
-      <c r="C93" s="0" t="s">
+      <c r="D93" s="0" t="s">
         <v>241</v>
-      </c>
-      <c r="D93" s="0" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>243</v>
       </c>
       <c r="D94" s="0" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C95" s="0" t="s">
         <v>245</v>
       </c>
       <c r="D95" s="0" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C96" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D96" s="0" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="s">
+        <v>250</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D97" s="0" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D98" s="0" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="s">
+        <v>256</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D99" s="0" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C100" s="0" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D100" s="0" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="s">
-        <v>256</v>
-      </c>
-      <c r="C101" s="0" t="s">
-        <v>257</v>
-      </c>
-      <c r="D101" s="0" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="0" t="s">
-        <v>259</v>
-      </c>
-      <c r="C102" s="0" t="s">
-        <v>260</v>
-      </c>
-      <c r="D102" s="0" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0" t="s">
         <v>262</v>
       </c>
-      <c r="C103" s="0" t="s">
+      <c r="C101" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D103" s="0" t="s">
+      <c r="D101" s="2" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="0" t="s">
-        <v>265</v>
-      </c>
-      <c r="C104" s="0" t="s">
-        <v>266</v>
-      </c>
-      <c r="D104" s="0" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="0" t="s">
-        <v>268</v>
-      </c>
-      <c r="C105" s="0" t="s">
-        <v>269</v>
-      </c>
-      <c r="D105" s="0" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="0" t="s">
-        <v>271</v>
-      </c>
-      <c r="C106" s="0" t="s">
-        <v>272</v>
-      </c>
-      <c r="D106" s="0" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0" t="s">
-        <v>274</v>
-      </c>
-      <c r="C107" s="0" t="s">
-        <v>275</v>
-      </c>
-      <c r="D107" s="0" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0" t="s">
-        <v>277</v>
-      </c>
-      <c r="C108" s="0" t="s">
-        <v>278</v>
-      </c>
-      <c r="D108" s="0" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="0" t="s">
-        <v>280</v>
-      </c>
-      <c r="C109" s="0" t="s">
-        <v>281</v>
-      </c>
-      <c r="D109" s="0" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0" t="s">
-        <v>283</v>
-      </c>
-      <c r="C110" s="0" t="s">
-        <v>284</v>
-      </c>
-      <c r="D110" s="0" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0" t="s">
-        <v>285</v>
-      </c>
-      <c r="C111" s="0" t="s">
-        <v>286</v>
-      </c>
-      <c r="D111" s="0" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0" t="s">
-        <v>288</v>
-      </c>
-      <c r="C112" s="0" t="s">
-        <v>289</v>
-      </c>
-      <c r="D112" s="0" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0" t="s">
-        <v>291</v>
-      </c>
-      <c r="C113" s="0" t="s">
-        <v>292</v>
-      </c>
-      <c r="D113" s="0" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="0" t="s">
-        <v>293</v>
-      </c>
-      <c r="C114" s="0" t="s">
-        <v>294</v>
-      </c>
-      <c r="D114" s="0" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="0" t="s">
-        <v>295</v>
-      </c>
-      <c r="C115" s="0" t="s">
-        <v>296</v>
-      </c>
-      <c r="D115" s="0" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="0" t="s">
-        <v>297</v>
-      </c>
-      <c r="C116" s="0" t="s">
-        <v>298</v>
-      </c>
-      <c r="D116" s="0" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="0" t="s">
-        <v>299</v>
-      </c>
-      <c r="C117" s="0" t="s">
-        <v>300</v>
-      </c>
-      <c r="D117" s="0" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="0" t="s">
-        <v>302</v>
-      </c>
-      <c r="C118" s="0" t="s">
-        <v>302</v>
-      </c>
-      <c r="D118" s="0" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="0" t="s">
-        <v>304</v>
-      </c>
-      <c r="C119" s="0" t="s">
-        <v>305</v>
-      </c>
-      <c r="D119" s="0" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="0" t="s">
-        <v>306</v>
-      </c>
-      <c r="C120" s="0" t="s">
-        <v>307</v>
-      </c>
-      <c r="D120" s="0" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="0" t="s">
-        <v>309</v>
-      </c>
-      <c r="C121" s="0" t="s">
-        <v>310</v>
-      </c>
-      <c r="D121" s="0" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="0" t="s">
-        <v>312</v>
-      </c>
-      <c r="C122" s="0" t="s">
-        <v>313</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="0" t="s">
-        <v>315</v>
-      </c>
-      <c r="C123" s="0" t="s">
-        <v>316</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="0" t="s">
-        <v>318</v>
-      </c>
-      <c r="C124" s="0" t="s">
-        <v>319</v>
-      </c>
-      <c r="D124" s="0" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="0" t="s">
-        <v>321</v>
-      </c>
-      <c r="C125" s="0" t="s">
-        <v>322</v>
-      </c>
-      <c r="D125" s="0" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="0" t="s">
-        <v>324</v>
-      </c>
-      <c r="C126" s="0" t="s">
-        <v>325</v>
-      </c>
-      <c r="D126" s="0" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="0" t="s">
-        <v>327</v>
-      </c>
-      <c r="C127" s="0" t="s">
-        <v>328</v>
-      </c>
-      <c r="D127" s="0" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="0" t="s">
-        <v>330</v>
-      </c>
-      <c r="C128" s="0" t="s">
-        <v>330</v>
-      </c>
-      <c r="D128" s="0" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="0" t="s">
-        <v>332</v>
-      </c>
-      <c r="C129" s="0" t="s">
-        <v>333</v>
-      </c>
-      <c r="D129" s="0" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="C130" s="0" t="s">
-        <v>336</v>
-      </c>
-      <c r="D130" s="0" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="0" t="s">
-        <v>338</v>
-      </c>
-      <c r="C131" s="0" t="s">
-        <v>339</v>
-      </c>
-      <c r="D131" s="0" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="C132" s="0" t="s">
-        <v>342</v>
-      </c>
-      <c r="D132" s="0" t="s">
-        <v>343</v>
-      </c>
-    </row>
+    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>